<commit_message>
finalized scripts for public repository (removed 'negative' from title, added session info, removed comments with test runs), added overview of R packages and versions, updated codebook for emolive study (occasions_total was missing), updated codebooks for simulation and aggregated results
</commit_message>
<xml_diff>
--- a/prepared data/emolive_codebook_benchmark_data.xlsx
+++ b/prepared data/emolive_codebook_benchmark_data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B34E613-82A2-4497-90E9-50B86E4AFF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D99782-A298-46D7-A3EC-3F47A200F711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4005" yWindow="7995" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="70">
   <si>
     <t>SERIAL</t>
   </si>
@@ -228,6 +228,12 @@
   </si>
   <si>
     <t>self-assured</t>
+  </si>
+  <si>
+    <t>occasion_total</t>
+  </si>
+  <si>
+    <t>number of total measurement occasion per participant (OVERALL occasions, not only valid)</t>
   </si>
 </sst>
 </file>
@@ -580,23 +586,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" customWidth="1"/>
-    <col min="2" max="2" width="41.5703125" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
-    <col min="4" max="4" width="35.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.33203125" customWidth="1"/>
+    <col min="2" max="2" width="41.5546875" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -610,13 +616,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -626,13 +632,13 @@
       <c r="C5" s="7"/>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -643,308 +649,317 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="C10" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C11" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="C12" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>15</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="C13" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>17</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="C14" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>19</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="C15" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>21</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="C16" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>23</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="C17" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>25</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="C18" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>27</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="C19" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>29</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="C20" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>31</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="C21" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>33</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="C22" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>35</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="C23" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>43</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="C24" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>44</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="C25" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>45</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="C26" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>46</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="C27" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>47</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="C28" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>48</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="C29" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>49</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="C30" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>50</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="C31" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>51</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="C32" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>52</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>65</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="C33" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
         <v>53</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="C34" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>54</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="7"/>
+      <c r="C35" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C36" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>